<commit_message>
Update: card and maptile back synced
</commit_message>
<xml_diff>
--- a/tts_envs/data/tokens.xlsx
+++ b/tts_envs/data/tokens.xlsx
@@ -5205,12 +5205,32 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>token_template</t>
+          <t>enemy_meeple_template</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
           <t>token</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>enemy Ant</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/cdenq/tts-roam-mod/main/assets/meeples/enemies/enemy_ant.png</t>
         </is>
       </c>
     </row>
@@ -5222,12 +5242,32 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>token_template</t>
+          <t>enemy_meeple_template</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
           <t>token</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>enemy Stag Beetle</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/cdenq/tts-roam-mod/main/assets/meeples/enemies/enemy_stagbeetle.png</t>
         </is>
       </c>
     </row>
@@ -5239,12 +5279,32 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>token_template</t>
+          <t>enemy_meeple_template</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
           <t>token</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>enemy Spider</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/cdenq/tts-roam-mod/main/assets/meeples/enemies/enemy_spider.png</t>
         </is>
       </c>
     </row>
@@ -5256,12 +5316,32 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>token_template</t>
+          <t>enemy_meeple_template</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
           <t>token</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>enemy Scorpion</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/cdenq/tts-roam-mod/main/assets/meeples/enemies/enemy_scorpion.png</t>
         </is>
       </c>
     </row>
@@ -5273,12 +5353,32 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>token_template</t>
+          <t>enemy_meeple_template</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
           <t>token</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>enemy Mantis</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/cdenq/tts-roam-mod/main/assets/meeples/enemies/enemy_mantis.png</t>
         </is>
       </c>
     </row>
@@ -5290,12 +5390,32 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>token_template</t>
+          <t>enemy_meeple_template</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
           <t>token</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>enemy Antlion</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/cdenq/tts-roam-mod/main/assets/meeples/enemies/enemy_antlion.png</t>
         </is>
       </c>
     </row>
@@ -5307,12 +5427,32 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>token_template</t>
+          <t>enemy_meeple_template</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
           <t>token</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>enemy Wasp</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/cdenq/tts-roam-mod/main/assets/meeples/enemies/enemy_wasp.png</t>
         </is>
       </c>
     </row>
@@ -5324,12 +5464,32 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>token_template</t>
+          <t>enemy_meeple_template</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
           <t>token</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>enemy Mosquito</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/cdenq/tts-roam-mod/main/assets/meeples/enemies/enemy_mosquito.png</t>
         </is>
       </c>
     </row>

</xml_diff>